<commit_message>
tabale enum end key
</commit_message>
<xml_diff>
--- a/Excels/Character.xlsx
+++ b/Excels/Character.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t xml:space="preserve">## 테이블 설명</t>
   </si>
@@ -53,6 +53,18 @@
   </si>
   <si>
     <t xml:space="preserve">Monster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[/enum]</t>
   </si>
   <si>
     <t xml:space="preserve">@dictionary</t>
@@ -366,28 +378,44 @@
       <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -395,10 +423,10 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>8</v>
@@ -415,10 +443,10 @@
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>6</v>
@@ -427,7 +455,7 @@
         <v>5</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -435,10 +463,10 @@
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>10</v>

</xml_diff>